<commit_message>
Ran grouping script after age_old annotation
</commit_message>
<xml_diff>
--- a/0-assets/raw_data/main/3-grouping/grouped_subreddit_data/quarterly_statistics.xlsx
+++ b/0-assets/raw_data/main/3-grouping/grouped_subreddit_data/quarterly_statistics.xlsx
@@ -721,13 +721,13 @@
         <v>142</v>
       </c>
       <c r="C10" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="D10" t="n">
         <v>53</v>
       </c>
       <c r="E10" t="n">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="F10" t="n">
         <v>4</v>
@@ -752,13 +752,13 @@
         <v>252</v>
       </c>
       <c r="C11" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="E11" t="n">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="F11" t="n">
         <v>16</v>
@@ -783,13 +783,13 @@
         <v>486</v>
       </c>
       <c r="C12" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>370</v>
+        <v>379</v>
       </c>
       <c r="E12" t="n">
-        <v>865</v>
+        <v>872</v>
       </c>
       <c r="F12" t="n">
         <v>28</v>
@@ -814,13 +814,13 @@
         <v>779</v>
       </c>
       <c r="C13" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>510</v>
+        <v>520</v>
       </c>
       <c r="E13" t="n">
-        <v>1206</v>
+        <v>1210</v>
       </c>
       <c r="F13" t="n">
         <v>42</v>
@@ -845,13 +845,13 @@
         <v>982</v>
       </c>
       <c r="C14" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>861</v>
+        <v>872</v>
       </c>
       <c r="E14" t="n">
-        <v>1489</v>
+        <v>1491</v>
       </c>
       <c r="F14" t="n">
         <v>18</v>
@@ -876,13 +876,13 @@
         <v>1195</v>
       </c>
       <c r="C15" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>1419</v>
+        <v>1432</v>
       </c>
       <c r="E15" t="n">
-        <v>1464</v>
+        <v>1473</v>
       </c>
       <c r="F15" t="n">
         <v>14</v>
@@ -907,13 +907,13 @@
         <v>3577</v>
       </c>
       <c r="C16" t="n">
-        <v>32</v>
+        <v>2</v>
       </c>
       <c r="D16" t="n">
-        <v>2080</v>
+        <v>2109</v>
       </c>
       <c r="E16" t="n">
-        <v>1289</v>
+        <v>1306</v>
       </c>
       <c r="F16" t="n">
         <v>18</v>
@@ -938,13 +938,13 @@
         <v>5793</v>
       </c>
       <c r="C17" t="n">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="D17" t="n">
-        <v>2355</v>
+        <v>2389</v>
       </c>
       <c r="E17" t="n">
-        <v>1455</v>
+        <v>1481</v>
       </c>
       <c r="F17" t="n">
         <v>22</v>
@@ -969,13 +969,13 @@
         <v>5595</v>
       </c>
       <c r="C18" t="n">
-        <v>74</v>
+        <v>25</v>
       </c>
       <c r="D18" t="n">
-        <v>2947</v>
+        <v>2992</v>
       </c>
       <c r="E18" t="n">
-        <v>1666</v>
+        <v>1687</v>
       </c>
       <c r="F18" t="n">
         <v>12</v>
@@ -1000,13 +1000,13 @@
         <v>4471</v>
       </c>
       <c r="C19" t="n">
-        <v>63</v>
+        <v>22</v>
       </c>
       <c r="D19" t="n">
-        <v>2593</v>
+        <v>2666</v>
       </c>
       <c r="E19" t="n">
-        <v>1728</v>
+        <v>1772</v>
       </c>
       <c r="F19" t="n">
         <v>9</v>
@@ -1031,13 +1031,13 @@
         <v>4278</v>
       </c>
       <c r="C20" t="n">
-        <v>68</v>
+        <v>22</v>
       </c>
       <c r="D20" t="n">
-        <v>2568</v>
+        <v>2702</v>
       </c>
       <c r="E20" t="n">
-        <v>1889</v>
+        <v>1983</v>
       </c>
       <c r="F20" t="n">
         <v>4</v>
@@ -1062,13 +1062,13 @@
         <v>2464</v>
       </c>
       <c r="C21" t="n">
-        <v>80</v>
+        <v>20</v>
       </c>
       <c r="D21" t="n">
-        <v>2169</v>
+        <v>2293</v>
       </c>
       <c r="E21" t="n">
-        <v>1762</v>
+        <v>1886</v>
       </c>
       <c r="F21" t="n">
         <v>4</v>
@@ -1093,13 +1093,13 @@
         <v>2433</v>
       </c>
       <c r="C22" t="n">
-        <v>74</v>
+        <v>23</v>
       </c>
       <c r="D22" t="n">
-        <v>2005</v>
+        <v>2118</v>
       </c>
       <c r="E22" t="n">
-        <v>2218</v>
+        <v>2328</v>
       </c>
       <c r="F22" t="n">
         <v>4</v>
@@ -1124,13 +1124,13 @@
         <v>1785</v>
       </c>
       <c r="C23" t="n">
-        <v>91</v>
+        <v>27</v>
       </c>
       <c r="D23" t="n">
-        <v>1937</v>
+        <v>2002</v>
       </c>
       <c r="E23" t="n">
-        <v>2314</v>
+        <v>2342</v>
       </c>
       <c r="F23" t="n">
         <v>5</v>
@@ -1155,13 +1155,13 @@
         <v>1778</v>
       </c>
       <c r="C24" t="n">
-        <v>99</v>
+        <v>26</v>
       </c>
       <c r="D24" t="n">
-        <v>1951</v>
+        <v>2032</v>
       </c>
       <c r="E24" t="n">
-        <v>2166</v>
+        <v>2228</v>
       </c>
       <c r="F24" t="n">
         <v>12</v>
@@ -1186,13 +1186,13 @@
         <v>1487</v>
       </c>
       <c r="C25" t="n">
-        <v>103</v>
+        <v>38</v>
       </c>
       <c r="D25" t="n">
-        <v>1592</v>
+        <v>1663</v>
       </c>
       <c r="E25" t="n">
-        <v>2145</v>
+        <v>2172</v>
       </c>
       <c r="F25" t="n">
         <v>12</v>
@@ -1217,13 +1217,13 @@
         <v>1449</v>
       </c>
       <c r="C26" t="n">
-        <v>182</v>
+        <v>61</v>
       </c>
       <c r="D26" t="n">
-        <v>1755</v>
+        <v>1805</v>
       </c>
       <c r="E26" t="n">
-        <v>2008</v>
+        <v>2042</v>
       </c>
       <c r="F26" t="n">
         <v>56</v>
@@ -1248,13 +1248,13 @@
         <v>1347</v>
       </c>
       <c r="C27" t="n">
-        <v>215</v>
+        <v>51</v>
       </c>
       <c r="D27" t="n">
-        <v>1728</v>
+        <v>1812</v>
       </c>
       <c r="E27" t="n">
-        <v>2068</v>
+        <v>2130</v>
       </c>
       <c r="F27" t="n">
         <v>76</v>
@@ -1279,13 +1279,13 @@
         <v>1927</v>
       </c>
       <c r="C28" t="n">
-        <v>240</v>
+        <v>88</v>
       </c>
       <c r="D28" t="n">
-        <v>1743</v>
+        <v>1835</v>
       </c>
       <c r="E28" t="n">
-        <v>1932</v>
+        <v>2013</v>
       </c>
       <c r="F28" t="n">
         <v>145</v>
@@ -1310,13 +1310,13 @@
         <v>1269</v>
       </c>
       <c r="C29" t="n">
-        <v>195</v>
+        <v>74</v>
       </c>
       <c r="D29" t="n">
-        <v>1755</v>
+        <v>1829</v>
       </c>
       <c r="E29" t="n">
-        <v>1787</v>
+        <v>1845</v>
       </c>
       <c r="F29" t="n">
         <v>187</v>
@@ -1341,13 +1341,13 @@
         <v>1532</v>
       </c>
       <c r="C30" t="n">
-        <v>228</v>
+        <v>75</v>
       </c>
       <c r="D30" t="n">
-        <v>1709</v>
+        <v>1785</v>
       </c>
       <c r="E30" t="n">
-        <v>1948</v>
+        <v>2007</v>
       </c>
       <c r="F30" t="n">
         <v>464</v>
@@ -1372,13 +1372,13 @@
         <v>1064</v>
       </c>
       <c r="C31" t="n">
-        <v>207</v>
+        <v>57</v>
       </c>
       <c r="D31" t="n">
-        <v>1809</v>
+        <v>1867</v>
       </c>
       <c r="E31" t="n">
-        <v>1872</v>
+        <v>1912</v>
       </c>
       <c r="F31" t="n">
         <v>117</v>
@@ -1403,13 +1403,13 @@
         <v>945</v>
       </c>
       <c r="C32" t="n">
-        <v>189</v>
+        <v>64</v>
       </c>
       <c r="D32" t="n">
-        <v>1730</v>
+        <v>1794</v>
       </c>
       <c r="E32" t="n">
-        <v>1722</v>
+        <v>1771</v>
       </c>
       <c r="F32" t="n">
         <v>30</v>
@@ -1434,13 +1434,13 @@
         <v>965</v>
       </c>
       <c r="C33" t="n">
-        <v>249</v>
+        <v>88</v>
       </c>
       <c r="D33" t="n">
-        <v>1829</v>
+        <v>1913</v>
       </c>
       <c r="E33" t="n">
-        <v>1644</v>
+        <v>1692</v>
       </c>
       <c r="F33" t="n">
         <v>21</v>
@@ -1465,13 +1465,13 @@
         <v>992</v>
       </c>
       <c r="C34" t="n">
-        <v>316</v>
+        <v>113</v>
       </c>
       <c r="D34" t="n">
-        <v>1531</v>
+        <v>1689</v>
       </c>
       <c r="E34" t="n">
-        <v>1738</v>
+        <v>1888</v>
       </c>
       <c r="F34" t="n">
         <v>191</v>
@@ -1496,13 +1496,13 @@
         <v>686</v>
       </c>
       <c r="C35" t="n">
-        <v>451</v>
+        <v>178</v>
       </c>
       <c r="D35" t="n">
-        <v>1699</v>
+        <v>2151</v>
       </c>
       <c r="E35" t="n">
-        <v>1835</v>
+        <v>2278</v>
       </c>
       <c r="F35" t="n">
         <v>380</v>
@@ -1527,13 +1527,13 @@
         <v>1162</v>
       </c>
       <c r="C36" t="n">
-        <v>486</v>
+        <v>204</v>
       </c>
       <c r="D36" t="n">
-        <v>1671</v>
+        <v>1966</v>
       </c>
       <c r="E36" t="n">
-        <v>1472</v>
+        <v>1747</v>
       </c>
       <c r="F36" t="n">
         <v>405</v>
@@ -1558,13 +1558,13 @@
         <v>1710</v>
       </c>
       <c r="C37" t="n">
-        <v>734</v>
+        <v>317</v>
       </c>
       <c r="D37" t="n">
-        <v>1783</v>
+        <v>1980</v>
       </c>
       <c r="E37" t="n">
-        <v>1277</v>
+        <v>1469</v>
       </c>
       <c r="F37" t="n">
         <v>413</v>
@@ -1589,13 +1589,13 @@
         <v>3563</v>
       </c>
       <c r="C38" t="n">
-        <v>755</v>
+        <v>314</v>
       </c>
       <c r="D38" t="n">
-        <v>1808</v>
+        <v>2064</v>
       </c>
       <c r="E38" t="n">
-        <v>1234</v>
+        <v>1480</v>
       </c>
       <c r="F38" t="n">
         <v>368</v>
@@ -1620,13 +1620,13 @@
         <v>5727</v>
       </c>
       <c r="C39" t="n">
-        <v>724</v>
+        <v>342</v>
       </c>
       <c r="D39" t="n">
-        <v>1726</v>
+        <v>1956</v>
       </c>
       <c r="E39" t="n">
-        <v>2937</v>
+        <v>3160</v>
       </c>
       <c r="F39" t="n">
         <v>264</v>
@@ -1651,13 +1651,13 @@
         <v>6817</v>
       </c>
       <c r="C40" t="n">
-        <v>739</v>
+        <v>327</v>
       </c>
       <c r="D40" t="n">
-        <v>1648</v>
+        <v>2168</v>
       </c>
       <c r="E40" t="n">
-        <v>3699</v>
+        <v>4210</v>
       </c>
       <c r="F40" t="n">
         <v>324</v>
@@ -1679,16 +1679,16 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>5699</v>
+        <v>5700</v>
       </c>
       <c r="C41" t="n">
-        <v>947</v>
+        <v>409</v>
       </c>
       <c r="D41" t="n">
-        <v>1636</v>
+        <v>2411</v>
       </c>
       <c r="E41" t="n">
-        <v>3559</v>
+        <v>4331</v>
       </c>
       <c r="F41" t="n">
         <v>395</v>
@@ -1713,13 +1713,13 @@
         <v>4946</v>
       </c>
       <c r="C42" t="n">
-        <v>935</v>
+        <v>435</v>
       </c>
       <c r="D42" t="n">
-        <v>1577</v>
+        <v>2388</v>
       </c>
       <c r="E42" t="n">
-        <v>3635</v>
+        <v>4442</v>
       </c>
       <c r="F42" t="n">
         <v>422</v>
@@ -1741,16 +1741,16 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>6376</v>
+        <v>6377</v>
       </c>
       <c r="C43" t="n">
-        <v>1041</v>
+        <v>516</v>
       </c>
       <c r="D43" t="n">
-        <v>1604</v>
+        <v>2459</v>
       </c>
       <c r="E43" t="n">
-        <v>3795</v>
+        <v>4646</v>
       </c>
       <c r="F43" t="n">
         <v>618</v>
@@ -1772,16 +1772,16 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>6141</v>
+        <v>6142</v>
       </c>
       <c r="C44" t="n">
-        <v>1411</v>
+        <v>762</v>
       </c>
       <c r="D44" t="n">
-        <v>2051</v>
+        <v>2782</v>
       </c>
       <c r="E44" t="n">
-        <v>3909</v>
+        <v>4637</v>
       </c>
       <c r="F44" t="n">
         <v>623</v>
@@ -1806,13 +1806,13 @@
         <v>4557</v>
       </c>
       <c r="C45" t="n">
-        <v>1339</v>
+        <v>719</v>
       </c>
       <c r="D45" t="n">
-        <v>1899</v>
+        <v>2406</v>
       </c>
       <c r="E45" t="n">
-        <v>3006</v>
+        <v>3502</v>
       </c>
       <c r="F45" t="n">
         <v>647</v>
@@ -1837,13 +1837,13 @@
         <v>4165</v>
       </c>
       <c r="C46" t="n">
-        <v>1336</v>
+        <v>729</v>
       </c>
       <c r="D46" t="n">
-        <v>2099</v>
+        <v>2547</v>
       </c>
       <c r="E46" t="n">
-        <v>3530</v>
+        <v>3956</v>
       </c>
       <c r="F46" t="n">
         <v>323</v>
@@ -1868,13 +1868,13 @@
         <v>4994</v>
       </c>
       <c r="C47" t="n">
-        <v>1613</v>
+        <v>931</v>
       </c>
       <c r="D47" t="n">
-        <v>2385</v>
+        <v>2981</v>
       </c>
       <c r="E47" t="n">
-        <v>3830</v>
+        <v>4408</v>
       </c>
       <c r="F47" t="n">
         <v>261</v>
@@ -1899,13 +1899,13 @@
         <v>6171</v>
       </c>
       <c r="C48" t="n">
-        <v>1582</v>
+        <v>692</v>
       </c>
       <c r="D48" t="n">
-        <v>2643</v>
+        <v>3236</v>
       </c>
       <c r="E48" t="n">
-        <v>4082</v>
+        <v>4634</v>
       </c>
       <c r="F48" t="n">
         <v>270</v>
@@ -1941,7 +1941,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-10-06T14:46:01</t>
+          <t>2026-10-07T22:15:35</t>
         </is>
       </c>
     </row>
@@ -1977,7 +1977,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0h 07m 48s</t>
+          <t>0h 07m 18s</t>
         </is>
       </c>
     </row>
@@ -2001,7 +2001,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0h 07m 49s</t>
+          <t>0h 07m 19s</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
age_young and age_old updated based on gender_male finds + cross-subreddit output moved
</commit_message>
<xml_diff>
--- a/0-assets/raw_data/main/3-grouping/grouped_subreddit_data/quarterly_statistics.xlsx
+++ b/0-assets/raw_data/main/3-grouping/grouped_subreddit_data/quarterly_statistics.xlsx
@@ -532,16 +532,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D4" t="n">
         <v>342</v>
       </c>
       <c r="E4" t="n">
-        <v>1282</v>
+        <v>1283</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
@@ -656,25 +656,25 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="C8" t="n">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="D8" t="n">
         <v>1409</v>
       </c>
       <c r="E8" t="n">
-        <v>2848</v>
+        <v>2864</v>
       </c>
       <c r="F8" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="G8" t="n">
         <v>519</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I8" t="n">
         <v>196</v>
@@ -687,25 +687,25 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>112</v>
+        <v>134</v>
       </c>
       <c r="C9" t="n">
-        <v>68</v>
+        <v>90</v>
       </c>
       <c r="D9" t="n">
         <v>1606</v>
       </c>
       <c r="E9" t="n">
-        <v>3222</v>
+        <v>3244</v>
       </c>
       <c r="F9" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G9" t="n">
         <v>766</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I9" t="n">
         <v>230</v>
@@ -724,10 +724,10 @@
         <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="E10" t="n">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="F10" t="n">
         <v>4</v>
@@ -755,19 +755,19 @@
         <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>141</v>
+        <v>107</v>
       </c>
       <c r="E11" t="n">
-        <v>375</v>
+        <v>403</v>
       </c>
       <c r="F11" t="n">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="G11" t="n">
         <v>7</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="I11" t="n">
         <v>55</v>
@@ -786,19 +786,19 @@
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>379</v>
+        <v>321</v>
       </c>
       <c r="E12" t="n">
-        <v>874</v>
+        <v>1021</v>
       </c>
       <c r="F12" t="n">
-        <v>28</v>
+        <v>71</v>
       </c>
       <c r="G12" t="n">
         <v>7</v>
       </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="I12" t="n">
         <v>38</v>
@@ -811,25 +811,25 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>779</v>
+        <v>780</v>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>520</v>
+        <v>434</v>
       </c>
       <c r="E13" t="n">
-        <v>1216</v>
+        <v>1490</v>
       </c>
       <c r="F13" t="n">
-        <v>42</v>
+        <v>123</v>
       </c>
       <c r="G13" t="n">
         <v>10</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="I13" t="n">
         <v>51</v>
@@ -842,25 +842,25 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>982</v>
+        <v>988</v>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D14" t="n">
-        <v>872</v>
+        <v>716</v>
       </c>
       <c r="E14" t="n">
-        <v>1500</v>
+        <v>2050</v>
       </c>
       <c r="F14" t="n">
-        <v>18</v>
+        <v>207</v>
       </c>
       <c r="G14" t="n">
         <v>20</v>
       </c>
       <c r="H14" t="n">
-        <v>8</v>
+        <v>197</v>
       </c>
       <c r="I14" t="n">
         <v>68</v>
@@ -873,25 +873,25 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1195</v>
+        <v>1209</v>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D15" t="n">
-        <v>1432</v>
+        <v>1178</v>
       </c>
       <c r="E15" t="n">
-        <v>1477</v>
+        <v>2565</v>
       </c>
       <c r="F15" t="n">
-        <v>14</v>
+        <v>328</v>
       </c>
       <c r="G15" t="n">
         <v>23</v>
       </c>
       <c r="H15" t="n">
-        <v>50</v>
+        <v>364</v>
       </c>
       <c r="I15" t="n">
         <v>56</v>
@@ -904,25 +904,25 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>3577</v>
+        <v>3585</v>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D16" t="n">
-        <v>2109</v>
+        <v>1629</v>
       </c>
       <c r="E16" t="n">
-        <v>1318</v>
+        <v>3145</v>
       </c>
       <c r="F16" t="n">
-        <v>18</v>
+        <v>520</v>
       </c>
       <c r="G16" t="n">
         <v>15</v>
       </c>
       <c r="H16" t="n">
-        <v>63</v>
+        <v>567</v>
       </c>
       <c r="I16" t="n">
         <v>74</v>
@@ -935,25 +935,25 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>5793</v>
+        <v>5820</v>
       </c>
       <c r="C17" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D17" t="n">
-        <v>2389</v>
+        <v>1887</v>
       </c>
       <c r="E17" t="n">
-        <v>1489</v>
+        <v>3664</v>
       </c>
       <c r="F17" t="n">
-        <v>22</v>
+        <v>675</v>
       </c>
       <c r="G17" t="n">
         <v>13</v>
       </c>
       <c r="H17" t="n">
-        <v>95</v>
+        <v>754</v>
       </c>
       <c r="I17" t="n">
         <v>71</v>
@@ -966,25 +966,25 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>5595</v>
+        <v>5629</v>
       </c>
       <c r="C18" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D18" t="n">
-        <v>2992</v>
+        <v>2395</v>
       </c>
       <c r="E18" t="n">
-        <v>1711</v>
+        <v>4478</v>
       </c>
       <c r="F18" t="n">
-        <v>12</v>
+        <v>750</v>
       </c>
       <c r="G18" t="n">
         <v>25</v>
       </c>
       <c r="H18" t="n">
-        <v>119</v>
+        <v>862</v>
       </c>
       <c r="I18" t="n">
         <v>82</v>
@@ -997,25 +997,25 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>4471</v>
+        <v>4502</v>
       </c>
       <c r="C19" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D19" t="n">
-        <v>2666</v>
+        <v>2123</v>
       </c>
       <c r="E19" t="n">
-        <v>1801</v>
+        <v>4211</v>
       </c>
       <c r="F19" t="n">
-        <v>9</v>
+        <v>613</v>
       </c>
       <c r="G19" t="n">
         <v>30</v>
       </c>
       <c r="H19" t="n">
-        <v>140</v>
+        <v>753</v>
       </c>
       <c r="I19" t="n">
         <v>71</v>
@@ -1028,25 +1028,25 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>4278</v>
+        <v>4334</v>
       </c>
       <c r="C20" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D20" t="n">
-        <v>2702</v>
+        <v>2133</v>
       </c>
       <c r="E20" t="n">
-        <v>2023</v>
+        <v>4335</v>
       </c>
       <c r="F20" t="n">
-        <v>4</v>
+        <v>592</v>
       </c>
       <c r="G20" t="n">
         <v>33</v>
       </c>
       <c r="H20" t="n">
-        <v>245</v>
+        <v>845</v>
       </c>
       <c r="I20" t="n">
         <v>117</v>
@@ -1059,25 +1059,25 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>2464</v>
+        <v>2497</v>
       </c>
       <c r="C21" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D21" t="n">
-        <v>2293</v>
+        <v>1773</v>
       </c>
       <c r="E21" t="n">
-        <v>1886</v>
+        <v>3917</v>
       </c>
       <c r="F21" t="n">
-        <v>4</v>
+        <v>515</v>
       </c>
       <c r="G21" t="n">
         <v>28</v>
       </c>
       <c r="H21" t="n">
-        <v>228</v>
+        <v>755</v>
       </c>
       <c r="I21" t="n">
         <v>108</v>
@@ -1090,25 +1090,25 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>2433</v>
+        <v>2477</v>
       </c>
       <c r="C22" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D22" t="n">
-        <v>2118</v>
+        <v>1592</v>
       </c>
       <c r="E22" t="n">
-        <v>2331</v>
+        <v>4207</v>
       </c>
       <c r="F22" t="n">
-        <v>4</v>
+        <v>552</v>
       </c>
       <c r="G22" t="n">
         <v>38</v>
       </c>
       <c r="H22" t="n">
-        <v>245</v>
+        <v>805</v>
       </c>
       <c r="I22" t="n">
         <v>149</v>
@@ -1121,25 +1121,25 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1785</v>
+        <v>1823</v>
       </c>
       <c r="C23" t="n">
         <v>27</v>
       </c>
       <c r="D23" t="n">
-        <v>2002</v>
+        <v>1424</v>
       </c>
       <c r="E23" t="n">
-        <v>2379</v>
+        <v>4148</v>
       </c>
       <c r="F23" t="n">
-        <v>5</v>
+        <v>472</v>
       </c>
       <c r="G23" t="n">
         <v>110</v>
       </c>
       <c r="H23" t="n">
-        <v>251</v>
+        <v>733</v>
       </c>
       <c r="I23" t="n">
         <v>157</v>
@@ -1152,25 +1152,25 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1778</v>
+        <v>1827</v>
       </c>
       <c r="C24" t="n">
         <v>26</v>
       </c>
       <c r="D24" t="n">
-        <v>2032</v>
+        <v>1495</v>
       </c>
       <c r="E24" t="n">
-        <v>2247</v>
+        <v>4016</v>
       </c>
       <c r="F24" t="n">
-        <v>12</v>
+        <v>469</v>
       </c>
       <c r="G24" t="n">
         <v>340</v>
       </c>
       <c r="H24" t="n">
-        <v>246</v>
+        <v>722</v>
       </c>
       <c r="I24" t="n">
         <v>174</v>
@@ -1183,25 +1183,25 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1487</v>
+        <v>1536</v>
       </c>
       <c r="C25" t="n">
         <v>38</v>
       </c>
       <c r="D25" t="n">
-        <v>1663</v>
+        <v>1206</v>
       </c>
       <c r="E25" t="n">
-        <v>2216</v>
+        <v>3657</v>
       </c>
       <c r="F25" t="n">
-        <v>12</v>
+        <v>400</v>
       </c>
       <c r="G25" t="n">
         <v>319</v>
       </c>
       <c r="H25" t="n">
-        <v>299</v>
+        <v>714</v>
       </c>
       <c r="I25" t="n">
         <v>202</v>
@@ -1214,25 +1214,25 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1449</v>
+        <v>1510</v>
       </c>
       <c r="C26" t="n">
         <v>61</v>
       </c>
       <c r="D26" t="n">
-        <v>1805</v>
+        <v>1364</v>
       </c>
       <c r="E26" t="n">
-        <v>2058</v>
+        <v>3736</v>
       </c>
       <c r="F26" t="n">
-        <v>56</v>
+        <v>559</v>
       </c>
       <c r="G26" t="n">
         <v>722</v>
       </c>
       <c r="H26" t="n">
-        <v>278</v>
+        <v>811</v>
       </c>
       <c r="I26" t="n">
         <v>193</v>
@@ -1245,25 +1245,25 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1347</v>
+        <v>1421</v>
       </c>
       <c r="C27" t="n">
         <v>51</v>
       </c>
       <c r="D27" t="n">
-        <v>1812</v>
+        <v>1285</v>
       </c>
       <c r="E27" t="n">
-        <v>2152</v>
+        <v>3793</v>
       </c>
       <c r="F27" t="n">
-        <v>76</v>
+        <v>568</v>
       </c>
       <c r="G27" t="n">
         <v>422</v>
       </c>
       <c r="H27" t="n">
-        <v>223</v>
+        <v>750</v>
       </c>
       <c r="I27" t="n">
         <v>282</v>
@@ -1276,25 +1276,25 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1927</v>
+        <v>1996</v>
       </c>
       <c r="C28" t="n">
         <v>88</v>
       </c>
       <c r="D28" t="n">
-        <v>1835</v>
+        <v>1311</v>
       </c>
       <c r="E28" t="n">
-        <v>2024</v>
+        <v>3702</v>
       </c>
       <c r="F28" t="n">
-        <v>145</v>
+        <v>595</v>
       </c>
       <c r="G28" t="n">
         <v>118</v>
       </c>
       <c r="H28" t="n">
-        <v>267</v>
+        <v>753</v>
       </c>
       <c r="I28" t="n">
         <v>267</v>
@@ -1307,25 +1307,25 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1269</v>
+        <v>1322</v>
       </c>
       <c r="C29" t="n">
         <v>74</v>
       </c>
       <c r="D29" t="n">
-        <v>1829</v>
+        <v>1198</v>
       </c>
       <c r="E29" t="n">
-        <v>1861</v>
+        <v>3533</v>
       </c>
       <c r="F29" t="n">
-        <v>187</v>
+        <v>770</v>
       </c>
       <c r="G29" t="n">
         <v>379</v>
       </c>
       <c r="H29" t="n">
-        <v>284</v>
+        <v>894</v>
       </c>
       <c r="I29" t="n">
         <v>288</v>
@@ -1338,25 +1338,25 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1532</v>
+        <v>1613</v>
       </c>
       <c r="C30" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D30" t="n">
-        <v>1785</v>
+        <v>1063</v>
       </c>
       <c r="E30" t="n">
-        <v>2024</v>
+        <v>3646</v>
       </c>
       <c r="F30" t="n">
-        <v>464</v>
+        <v>1003</v>
       </c>
       <c r="G30" t="n">
-        <v>459</v>
+        <v>514</v>
       </c>
       <c r="H30" t="n">
-        <v>271</v>
+        <v>830</v>
       </c>
       <c r="I30" t="n">
         <v>313</v>
@@ -1369,25 +1369,25 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1064</v>
+        <v>1138</v>
       </c>
       <c r="C31" t="n">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="D31" t="n">
-        <v>1867</v>
+        <v>915</v>
       </c>
       <c r="E31" t="n">
-        <v>1930</v>
+        <v>3657</v>
       </c>
       <c r="F31" t="n">
-        <v>117</v>
+        <v>695</v>
       </c>
       <c r="G31" t="n">
-        <v>506</v>
+        <v>572</v>
       </c>
       <c r="H31" t="n">
-        <v>312</v>
+        <v>925</v>
       </c>
       <c r="I31" t="n">
         <v>378</v>
@@ -1400,25 +1400,25 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>945</v>
+        <v>1024</v>
       </c>
       <c r="C32" t="n">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="D32" t="n">
-        <v>1794</v>
+        <v>847</v>
       </c>
       <c r="E32" t="n">
-        <v>1786</v>
+        <v>3422</v>
       </c>
       <c r="F32" t="n">
-        <v>30</v>
+        <v>575</v>
       </c>
       <c r="G32" t="n">
-        <v>552</v>
+        <v>626</v>
       </c>
       <c r="H32" t="n">
-        <v>309</v>
+        <v>891</v>
       </c>
       <c r="I32" t="n">
         <v>384</v>
@@ -1431,25 +1431,25 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>965</v>
+        <v>1089</v>
       </c>
       <c r="C33" t="n">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="D33" t="n">
-        <v>1913</v>
+        <v>814</v>
       </c>
       <c r="E33" t="n">
-        <v>1728</v>
+        <v>3430</v>
       </c>
       <c r="F33" t="n">
-        <v>21</v>
+        <v>609</v>
       </c>
       <c r="G33" t="n">
-        <v>665</v>
+        <v>750</v>
       </c>
       <c r="H33" t="n">
-        <v>330</v>
+        <v>957</v>
       </c>
       <c r="I33" t="n">
         <v>372</v>
@@ -1462,25 +1462,25 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>992</v>
+        <v>1131</v>
       </c>
       <c r="C34" t="n">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="D34" t="n">
-        <v>1689</v>
+        <v>781</v>
       </c>
       <c r="E34" t="n">
-        <v>1896</v>
+        <v>3331</v>
       </c>
       <c r="F34" t="n">
-        <v>191</v>
+        <v>664</v>
       </c>
       <c r="G34" t="n">
-        <v>764</v>
+        <v>835</v>
       </c>
       <c r="H34" t="n">
-        <v>249</v>
+        <v>774</v>
       </c>
       <c r="I34" t="n">
         <v>376</v>
@@ -1493,25 +1493,25 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>686</v>
+        <v>882</v>
       </c>
       <c r="C35" t="n">
-        <v>178</v>
+        <v>190</v>
       </c>
       <c r="D35" t="n">
-        <v>2151</v>
+        <v>912</v>
       </c>
       <c r="E35" t="n">
-        <v>2287</v>
+        <v>3858</v>
       </c>
       <c r="F35" t="n">
-        <v>380</v>
+        <v>841</v>
       </c>
       <c r="G35" t="n">
-        <v>858</v>
+        <v>908</v>
       </c>
       <c r="H35" t="n">
-        <v>359</v>
+        <v>902</v>
       </c>
       <c r="I35" t="n">
         <v>456</v>
@@ -1524,25 +1524,25 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1162</v>
+        <v>1383</v>
       </c>
       <c r="C36" t="n">
-        <v>204</v>
+        <v>211</v>
       </c>
       <c r="D36" t="n">
-        <v>1966</v>
+        <v>847</v>
       </c>
       <c r="E36" t="n">
-        <v>1767</v>
+        <v>3286</v>
       </c>
       <c r="F36" t="n">
-        <v>405</v>
+        <v>886</v>
       </c>
       <c r="G36" t="n">
-        <v>1084</v>
+        <v>1137</v>
       </c>
       <c r="H36" t="n">
-        <v>385</v>
+        <v>924</v>
       </c>
       <c r="I36" t="n">
         <v>362</v>
@@ -1555,25 +1555,25 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1710</v>
+        <v>2012</v>
       </c>
       <c r="C37" t="n">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="D37" t="n">
-        <v>1980</v>
+        <v>877</v>
       </c>
       <c r="E37" t="n">
-        <v>1474</v>
+        <v>3068</v>
       </c>
       <c r="F37" t="n">
-        <v>413</v>
+        <v>875</v>
       </c>
       <c r="G37" t="n">
-        <v>1039</v>
+        <v>1096</v>
       </c>
       <c r="H37" t="n">
-        <v>377</v>
+        <v>953</v>
       </c>
       <c r="I37" t="n">
         <v>294</v>
@@ -1586,25 +1586,25 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>3563</v>
+        <v>3882</v>
       </c>
       <c r="C38" t="n">
-        <v>314</v>
+        <v>320</v>
       </c>
       <c r="D38" t="n">
-        <v>2064</v>
+        <v>919</v>
       </c>
       <c r="E38" t="n">
-        <v>1490</v>
+        <v>3086</v>
       </c>
       <c r="F38" t="n">
-        <v>368</v>
+        <v>746</v>
       </c>
       <c r="G38" t="n">
-        <v>1061</v>
+        <v>1110</v>
       </c>
       <c r="H38" t="n">
-        <v>323</v>
+        <v>805</v>
       </c>
       <c r="I38" t="n">
         <v>328</v>
@@ -1617,28 +1617,28 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>5727</v>
+        <v>6054</v>
       </c>
       <c r="C39" t="n">
-        <v>342</v>
+        <v>363</v>
       </c>
       <c r="D39" t="n">
-        <v>1956</v>
+        <v>873</v>
       </c>
       <c r="E39" t="n">
-        <v>3167</v>
+        <v>4660</v>
       </c>
       <c r="F39" t="n">
-        <v>264</v>
+        <v>632</v>
       </c>
       <c r="G39" t="n">
-        <v>783</v>
+        <v>842</v>
       </c>
       <c r="H39" t="n">
-        <v>384</v>
+        <v>854</v>
       </c>
       <c r="I39" t="n">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="40">
@@ -1648,28 +1648,28 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>6817</v>
+        <v>7111</v>
       </c>
       <c r="C40" t="n">
-        <v>327</v>
+        <v>343</v>
       </c>
       <c r="D40" t="n">
-        <v>2168</v>
+        <v>936</v>
       </c>
       <c r="E40" t="n">
-        <v>4219</v>
+        <v>5693</v>
       </c>
       <c r="F40" t="n">
-        <v>324</v>
+        <v>651</v>
       </c>
       <c r="G40" t="n">
-        <v>882</v>
+        <v>974</v>
       </c>
       <c r="H40" t="n">
-        <v>389</v>
+        <v>793</v>
       </c>
       <c r="I40" t="n">
-        <v>333</v>
+        <v>340</v>
       </c>
     </row>
     <row r="41">
@@ -1679,28 +1679,28 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>5700</v>
+        <v>6091</v>
       </c>
       <c r="C41" t="n">
-        <v>409</v>
+        <v>430</v>
       </c>
       <c r="D41" t="n">
-        <v>2411</v>
+        <v>1203</v>
       </c>
       <c r="E41" t="n">
-        <v>4334</v>
+        <v>5727</v>
       </c>
       <c r="F41" t="n">
-        <v>395</v>
+        <v>700</v>
       </c>
       <c r="G41" t="n">
-        <v>875</v>
+        <v>938</v>
       </c>
       <c r="H41" t="n">
-        <v>352</v>
+        <v>738</v>
       </c>
       <c r="I41" t="n">
-        <v>511</v>
+        <v>518</v>
       </c>
     </row>
     <row r="42">
@@ -1710,28 +1710,28 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>4946</v>
+        <v>5288</v>
       </c>
       <c r="C42" t="n">
-        <v>435</v>
+        <v>454</v>
       </c>
       <c r="D42" t="n">
-        <v>2388</v>
+        <v>1145</v>
       </c>
       <c r="E42" t="n">
-        <v>4446</v>
+        <v>5781</v>
       </c>
       <c r="F42" t="n">
-        <v>422</v>
+        <v>729</v>
       </c>
       <c r="G42" t="n">
-        <v>896</v>
+        <v>948</v>
       </c>
       <c r="H42" t="n">
-        <v>300</v>
+        <v>686</v>
       </c>
       <c r="I42" t="n">
-        <v>471</v>
+        <v>473</v>
       </c>
     </row>
     <row r="43">
@@ -1741,28 +1741,28 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>6377</v>
+        <v>6751</v>
       </c>
       <c r="C43" t="n">
-        <v>516</v>
+        <v>537</v>
       </c>
       <c r="D43" t="n">
-        <v>2459</v>
+        <v>1196</v>
       </c>
       <c r="E43" t="n">
-        <v>4650</v>
+        <v>5857</v>
       </c>
       <c r="F43" t="n">
-        <v>618</v>
+        <v>910</v>
       </c>
       <c r="G43" t="n">
-        <v>644</v>
+        <v>721</v>
       </c>
       <c r="H43" t="n">
-        <v>88</v>
+        <v>458</v>
       </c>
       <c r="I43" t="n">
-        <v>370</v>
+        <v>381</v>
       </c>
     </row>
     <row r="44">
@@ -1772,28 +1772,28 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>6142</v>
+        <v>6582</v>
       </c>
       <c r="C44" t="n">
-        <v>762</v>
+        <v>788</v>
       </c>
       <c r="D44" t="n">
-        <v>2782</v>
+        <v>1219</v>
       </c>
       <c r="E44" t="n">
-        <v>4640</v>
+        <v>5984</v>
       </c>
       <c r="F44" t="n">
-        <v>623</v>
+        <v>904</v>
       </c>
       <c r="G44" t="n">
-        <v>755</v>
+        <v>815</v>
       </c>
       <c r="H44" t="n">
-        <v>60</v>
+        <v>443</v>
       </c>
       <c r="I44" t="n">
-        <v>348</v>
+        <v>359</v>
       </c>
     </row>
     <row r="45">
@@ -1803,28 +1803,28 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>4557</v>
+        <v>4987</v>
       </c>
       <c r="C45" t="n">
-        <v>719</v>
+        <v>740</v>
       </c>
       <c r="D45" t="n">
-        <v>2406</v>
+        <v>1002</v>
       </c>
       <c r="E45" t="n">
-        <v>3513</v>
+        <v>4806</v>
       </c>
       <c r="F45" t="n">
-        <v>647</v>
+        <v>887</v>
       </c>
       <c r="G45" t="n">
-        <v>868</v>
+        <v>933</v>
       </c>
       <c r="H45" t="n">
-        <v>48</v>
+        <v>368</v>
       </c>
       <c r="I45" t="n">
-        <v>326</v>
+        <v>342</v>
       </c>
     </row>
     <row r="46">
@@ -1834,28 +1834,28 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>4165</v>
+        <v>4604</v>
       </c>
       <c r="C46" t="n">
-        <v>729</v>
+        <v>762</v>
       </c>
       <c r="D46" t="n">
-        <v>2547</v>
+        <v>907</v>
       </c>
       <c r="E46" t="n">
-        <v>3978</v>
+        <v>5182</v>
       </c>
       <c r="F46" t="n">
-        <v>323</v>
+        <v>583</v>
       </c>
       <c r="G46" t="n">
-        <v>719</v>
+        <v>804</v>
       </c>
       <c r="H46" t="n">
-        <v>46</v>
+        <v>375</v>
       </c>
       <c r="I46" t="n">
-        <v>444</v>
+        <v>467</v>
       </c>
     </row>
     <row r="47">
@@ -1865,28 +1865,28 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>4994</v>
+        <v>5474</v>
       </c>
       <c r="C47" t="n">
-        <v>931</v>
+        <v>976</v>
       </c>
       <c r="D47" t="n">
-        <v>2981</v>
+        <v>1013</v>
       </c>
       <c r="E47" t="n">
-        <v>4426</v>
+        <v>5681</v>
       </c>
       <c r="F47" t="n">
-        <v>261</v>
+        <v>527</v>
       </c>
       <c r="G47" t="n">
-        <v>531</v>
+        <v>599</v>
       </c>
       <c r="H47" t="n">
-        <v>39</v>
+        <v>397</v>
       </c>
       <c r="I47" t="n">
-        <v>643</v>
+        <v>703</v>
       </c>
     </row>
     <row r="48">
@@ -1896,28 +1896,28 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>6171</v>
+        <v>6665</v>
       </c>
       <c r="C48" t="n">
-        <v>692</v>
+        <v>723</v>
       </c>
       <c r="D48" t="n">
-        <v>3236</v>
+        <v>1011</v>
       </c>
       <c r="E48" t="n">
-        <v>4675</v>
+        <v>6073</v>
       </c>
       <c r="F48" t="n">
-        <v>270</v>
+        <v>595</v>
       </c>
       <c r="G48" t="n">
-        <v>531</v>
+        <v>612</v>
       </c>
       <c r="H48" t="n">
-        <v>64</v>
+        <v>486</v>
       </c>
       <c r="I48" t="n">
-        <v>782</v>
+        <v>846</v>
       </c>
     </row>
   </sheetData>
@@ -1941,7 +1941,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-10-07T22:29:59</t>
+          <t>2026-10-08T19:04:25</t>
         </is>
       </c>
     </row>
@@ -1977,7 +1977,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0h 06m 42s</t>
+          <t>0h 06m 35s</t>
         </is>
       </c>
     </row>
@@ -2001,7 +2001,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0h 06m 43s</t>
+          <t>0h 06m 36s</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
gender_male updated after finds in female/diverse
</commit_message>
<xml_diff>
--- a/0-assets/raw_data/main/3-grouping/grouped_subreddit_data/quarterly_statistics.xlsx
+++ b/0-assets/raw_data/main/3-grouping/grouped_subreddit_data/quarterly_statistics.xlsx
@@ -532,13 +532,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D4" t="n">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="E4" t="n">
         <v>1283</v>
@@ -563,13 +563,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C5" t="n">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="D5" t="n">
-        <v>498</v>
+        <v>510</v>
       </c>
       <c r="E5" t="n">
         <v>1442</v>
@@ -594,13 +594,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="C6" t="n">
-        <v>13</v>
+        <v>78</v>
       </c>
       <c r="D6" t="n">
-        <v>669</v>
+        <v>734</v>
       </c>
       <c r="E6" t="n">
         <v>1816</v>
@@ -625,13 +625,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="C7" t="n">
-        <v>31</v>
+        <v>101</v>
       </c>
       <c r="D7" t="n">
-        <v>803</v>
+        <v>873</v>
       </c>
       <c r="E7" t="n">
         <v>2276</v>
@@ -656,13 +656,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>19</v>
+        <v>157</v>
       </c>
       <c r="C8" t="n">
-        <v>60</v>
+        <v>198</v>
       </c>
       <c r="D8" t="n">
-        <v>1409</v>
+        <v>1590</v>
       </c>
       <c r="E8" t="n">
         <v>2864</v>
@@ -671,13 +671,13 @@
         <v>19</v>
       </c>
       <c r="G8" t="n">
-        <v>519</v>
+        <v>531</v>
       </c>
       <c r="H8" t="n">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="I8" t="n">
-        <v>196</v>
+        <v>208</v>
       </c>
     </row>
     <row r="9">
@@ -687,13 +687,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>134</v>
+        <v>335</v>
       </c>
       <c r="C9" t="n">
-        <v>90</v>
+        <v>291</v>
       </c>
       <c r="D9" t="n">
-        <v>1606</v>
+        <v>1857</v>
       </c>
       <c r="E9" t="n">
         <v>3244</v>
@@ -702,13 +702,13 @@
         <v>25</v>
       </c>
       <c r="G9" t="n">
-        <v>766</v>
+        <v>774</v>
       </c>
       <c r="H9" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I9" t="n">
-        <v>230</v>
+        <v>238</v>
       </c>
     </row>
     <row r="10">
@@ -727,7 +727,7 @@
         <v>43</v>
       </c>
       <c r="E10" t="n">
-        <v>281</v>
+        <v>96</v>
       </c>
       <c r="F10" t="n">
         <v>4</v>
@@ -758,7 +758,7 @@
         <v>107</v>
       </c>
       <c r="E11" t="n">
-        <v>403</v>
+        <v>196</v>
       </c>
       <c r="F11" t="n">
         <v>27</v>
@@ -789,7 +789,7 @@
         <v>321</v>
       </c>
       <c r="E12" t="n">
-        <v>1021</v>
+        <v>504</v>
       </c>
       <c r="F12" t="n">
         <v>71</v>
@@ -820,7 +820,7 @@
         <v>434</v>
       </c>
       <c r="E13" t="n">
-        <v>1490</v>
+        <v>681</v>
       </c>
       <c r="F13" t="n">
         <v>123</v>
@@ -851,7 +851,7 @@
         <v>716</v>
       </c>
       <c r="E14" t="n">
-        <v>2050</v>
+        <v>918</v>
       </c>
       <c r="F14" t="n">
         <v>207</v>
@@ -882,7 +882,7 @@
         <v>1178</v>
       </c>
       <c r="E15" t="n">
-        <v>2565</v>
+        <v>1002</v>
       </c>
       <c r="F15" t="n">
         <v>328</v>
@@ -913,7 +913,7 @@
         <v>1629</v>
       </c>
       <c r="E16" t="n">
-        <v>3145</v>
+        <v>1168</v>
       </c>
       <c r="F16" t="n">
         <v>520</v>
@@ -944,7 +944,7 @@
         <v>1887</v>
       </c>
       <c r="E17" t="n">
-        <v>3664</v>
+        <v>1349</v>
       </c>
       <c r="F17" t="n">
         <v>675</v>
@@ -975,7 +975,7 @@
         <v>2395</v>
       </c>
       <c r="E18" t="n">
-        <v>4478</v>
+        <v>1566</v>
       </c>
       <c r="F18" t="n">
         <v>750</v>
@@ -1006,7 +1006,7 @@
         <v>2123</v>
       </c>
       <c r="E19" t="n">
-        <v>4211</v>
+        <v>1507</v>
       </c>
       <c r="F19" t="n">
         <v>613</v>
@@ -1037,7 +1037,7 @@
         <v>2133</v>
       </c>
       <c r="E20" t="n">
-        <v>4335</v>
+        <v>1643</v>
       </c>
       <c r="F20" t="n">
         <v>592</v>
@@ -1068,7 +1068,7 @@
         <v>1773</v>
       </c>
       <c r="E21" t="n">
-        <v>3917</v>
+        <v>1738</v>
       </c>
       <c r="F21" t="n">
         <v>515</v>
@@ -1099,7 +1099,7 @@
         <v>1592</v>
       </c>
       <c r="E22" t="n">
-        <v>4207</v>
+        <v>1911</v>
       </c>
       <c r="F22" t="n">
         <v>552</v>
@@ -1130,7 +1130,7 @@
         <v>1424</v>
       </c>
       <c r="E23" t="n">
-        <v>4148</v>
+        <v>1826</v>
       </c>
       <c r="F23" t="n">
         <v>472</v>
@@ -1161,7 +1161,7 @@
         <v>1495</v>
       </c>
       <c r="E24" t="n">
-        <v>4016</v>
+        <v>1711</v>
       </c>
       <c r="F24" t="n">
         <v>469</v>
@@ -1192,7 +1192,7 @@
         <v>1206</v>
       </c>
       <c r="E25" t="n">
-        <v>3657</v>
+        <v>1688</v>
       </c>
       <c r="F25" t="n">
         <v>400</v>
@@ -1223,7 +1223,7 @@
         <v>1364</v>
       </c>
       <c r="E26" t="n">
-        <v>3736</v>
+        <v>1713</v>
       </c>
       <c r="F26" t="n">
         <v>559</v>
@@ -1254,7 +1254,7 @@
         <v>1285</v>
       </c>
       <c r="E27" t="n">
-        <v>3793</v>
+        <v>1861</v>
       </c>
       <c r="F27" t="n">
         <v>568</v>
@@ -1285,7 +1285,7 @@
         <v>1311</v>
       </c>
       <c r="E28" t="n">
-        <v>3702</v>
+        <v>1782</v>
       </c>
       <c r="F28" t="n">
         <v>595</v>
@@ -1316,7 +1316,7 @@
         <v>1198</v>
       </c>
       <c r="E29" t="n">
-        <v>3533</v>
+        <v>1844</v>
       </c>
       <c r="F29" t="n">
         <v>770</v>
@@ -1347,7 +1347,7 @@
         <v>1063</v>
       </c>
       <c r="E30" t="n">
-        <v>3646</v>
+        <v>1734</v>
       </c>
       <c r="F30" t="n">
         <v>1003</v>
@@ -1378,7 +1378,7 @@
         <v>915</v>
       </c>
       <c r="E31" t="n">
-        <v>3657</v>
+        <v>1721</v>
       </c>
       <c r="F31" t="n">
         <v>695</v>
@@ -1409,7 +1409,7 @@
         <v>847</v>
       </c>
       <c r="E32" t="n">
-        <v>3422</v>
+        <v>1620</v>
       </c>
       <c r="F32" t="n">
         <v>575</v>
@@ -1440,7 +1440,7 @@
         <v>814</v>
       </c>
       <c r="E33" t="n">
-        <v>3430</v>
+        <v>1410</v>
       </c>
       <c r="F33" t="n">
         <v>609</v>
@@ -1471,7 +1471,7 @@
         <v>781</v>
       </c>
       <c r="E34" t="n">
-        <v>3331</v>
+        <v>1391</v>
       </c>
       <c r="F34" t="n">
         <v>664</v>
@@ -1502,7 +1502,7 @@
         <v>912</v>
       </c>
       <c r="E35" t="n">
-        <v>3858</v>
+        <v>1536</v>
       </c>
       <c r="F35" t="n">
         <v>841</v>
@@ -1533,7 +1533,7 @@
         <v>847</v>
       </c>
       <c r="E36" t="n">
-        <v>3286</v>
+        <v>1223</v>
       </c>
       <c r="F36" t="n">
         <v>886</v>
@@ -1564,7 +1564,7 @@
         <v>877</v>
       </c>
       <c r="E37" t="n">
-        <v>3068</v>
+        <v>1073</v>
       </c>
       <c r="F37" t="n">
         <v>875</v>
@@ -1595,7 +1595,7 @@
         <v>919</v>
       </c>
       <c r="E38" t="n">
-        <v>3086</v>
+        <v>1091</v>
       </c>
       <c r="F38" t="n">
         <v>746</v>
@@ -1626,7 +1626,7 @@
         <v>873</v>
       </c>
       <c r="E39" t="n">
-        <v>4660</v>
+        <v>2755</v>
       </c>
       <c r="F39" t="n">
         <v>632</v>
@@ -1657,7 +1657,7 @@
         <v>936</v>
       </c>
       <c r="E40" t="n">
-        <v>5693</v>
+        <v>3521</v>
       </c>
       <c r="F40" t="n">
         <v>651</v>
@@ -1688,7 +1688,7 @@
         <v>1203</v>
       </c>
       <c r="E41" t="n">
-        <v>5727</v>
+        <v>2715</v>
       </c>
       <c r="F41" t="n">
         <v>700</v>
@@ -1719,7 +1719,7 @@
         <v>1145</v>
       </c>
       <c r="E42" t="n">
-        <v>5781</v>
+        <v>2206</v>
       </c>
       <c r="F42" t="n">
         <v>729</v>
@@ -1750,7 +1750,7 @@
         <v>1196</v>
       </c>
       <c r="E43" t="n">
-        <v>5857</v>
+        <v>2336</v>
       </c>
       <c r="F43" t="n">
         <v>910</v>
@@ -1781,7 +1781,7 @@
         <v>1219</v>
       </c>
       <c r="E44" t="n">
-        <v>5984</v>
+        <v>2348</v>
       </c>
       <c r="F44" t="n">
         <v>904</v>
@@ -1812,7 +1812,7 @@
         <v>1002</v>
       </c>
       <c r="E45" t="n">
-        <v>4806</v>
+        <v>1702</v>
       </c>
       <c r="F45" t="n">
         <v>887</v>
@@ -1843,7 +1843,7 @@
         <v>907</v>
       </c>
       <c r="E46" t="n">
-        <v>5182</v>
+        <v>2256</v>
       </c>
       <c r="F46" t="n">
         <v>583</v>
@@ -1874,7 +1874,7 @@
         <v>1013</v>
       </c>
       <c r="E47" t="n">
-        <v>5681</v>
+        <v>2415</v>
       </c>
       <c r="F47" t="n">
         <v>527</v>
@@ -1905,7 +1905,7 @@
         <v>1011</v>
       </c>
       <c r="E48" t="n">
-        <v>6073</v>
+        <v>2922</v>
       </c>
       <c r="F48" t="n">
         <v>595</v>
@@ -1941,7 +1941,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-10-08T19:04:25</t>
+          <t>2026-10-09T19:42:24</t>
         </is>
       </c>
     </row>
@@ -1977,7 +1977,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0h 06m 35s</t>
+          <t>0h 06m 41s</t>
         </is>
       </c>
     </row>
@@ -2001,7 +2001,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0h 06m 36s</t>
+          <t>0h 06m 42s</t>
         </is>
       </c>
     </row>

</xml_diff>